<commit_message>
Refactor Excel handling with openpyxl, improve file reading and formatting
Co-authored-by: lars.bruurmijn <lars.bruurmijn@nl-grc.com>
</commit_message>
<xml_diff>
--- a/voorbeelden/norm_bestand_voorbeeld.xlsx
+++ b/voorbeelden/norm_bestand_voorbeeld.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,11 +455,6 @@
           <t>Complexiteit</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Norm_Beschrijving</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -485,11 +480,6 @@
           <t>Hoog</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Volledige projectmanagement inclusief planning en controle</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -515,11 +505,6 @@
           <t>Gemiddeld</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Uitgebreide data-analyse met rapportage en visualisatie</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -545,11 +530,6 @@
           <t>Laag</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Professionele documentcreatie volgens bedrijfsstandaarden</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -575,11 +555,6 @@
           <t>Laag</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Effectieve presentaties voor verschillende doelgroepen</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -603,11 +578,6 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>Gemiddeld</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Systematische kwaliteitscontrole en validatie processen</t>
         </is>
       </c>
     </row>

</xml_diff>